<commit_message>
Fix data validation and merging
</commit_message>
<xml_diff>
--- a/outputs/ranking.xlsx
+++ b/outputs/ranking.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xếp hạng Cách A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trụ cột Cách A" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhóm Cách A" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xếp hạng Cách B" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trụ cột Cách B" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhóm Cách B" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Độ vững" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dirichlet" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Xếp hạng Cách A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Trụ cột Cách A" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Nhóm Cách A" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Xếp hạng Cách B" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Trụ cột Cách B" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Nhóm Cách B" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Độ vững" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dirichlet" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,16 +24,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -44,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -52,21 +49,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,52 +424,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>DBI</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Hạng</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>DBI S1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Hạng S1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DBI S2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Hạng S2</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>DBI S3</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Hạng S3</t>
         </is>
@@ -682,44 +670,44 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>1. Trụ cột Khách hàng</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>2. Trụ cột Chiến lược</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>3. Trụ cột Công nghệ</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>4. Trụ cột Vận hành</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>5. Trụ cột Văn hóa</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>6. Trụ cột Dữ liệu</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -744,7 +732,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -769,7 +757,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -794,7 +782,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -819,7 +807,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>
@@ -858,139 +846,139 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -1070,7 +1058,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -1152,7 +1140,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -1234,7 +1222,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -1316,7 +1304,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>
@@ -1412,52 +1400,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>DBI</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Hạng</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>DBI S1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Hạng S1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DBI S2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Hạng S2</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>DBI S3</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Hạng S3</t>
         </is>
@@ -1658,44 +1646,44 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>1. Trụ cột Khách hàng</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>2. Trụ cột Chiến lược</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>3. Trụ cột Công nghệ</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>4. Trụ cột Vận hành</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>5. Trụ cột Văn hóa</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>6. Trụ cột Dữ liệu</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -1720,7 +1708,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -1745,7 +1733,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -1770,7 +1758,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -1795,7 +1783,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>
@@ -1834,139 +1822,139 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -2048,7 +2036,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -2130,7 +2118,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -2212,7 +2200,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -2294,7 +2282,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>
@@ -2390,27 +2378,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Cách</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Kịch bản</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Mô tả</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spearman vs cơ sở A</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Ngân hàng đổi hạng</t>
         </is>
@@ -2615,34 +2603,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Hạng 1 (%)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Hạng 2 (%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Hạng 3 (%)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Hạng 4 (%)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Hạng 5 (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -2664,7 +2652,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -2686,7 +2674,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -2708,7 +2696,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -2730,7 +2718,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>

</xml_diff>

<commit_message>
Update bank evidence and digital transformation ranking
</commit_message>
<xml_diff>
--- a/outputs/ranking.xlsx
+++ b/outputs/ranking.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Xếp hạng Cách A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Trụ cột Cách A" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Nhóm Cách A" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Xếp hạng Cách B" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Trụ cột Cách B" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Nhóm Cách B" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Độ vững" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Dirichlet" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xếp hạng Cách A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trụ cột Cách A" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhóm Cách A" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xếp hạng Cách B" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trụ cột Cách B" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhóm Cách B" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Độ vững" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dirichlet" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,13 +24,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +44,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,12 +52,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,52 +436,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>DBI</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Hạng</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>DBI S1</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Hạng S1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DBI S2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Hạng S2</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>DBI S3</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Hạng S3</t>
         </is>
@@ -670,44 +682,44 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1. Trụ cột Khách hàng</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>2. Trụ cột Chiến lược</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>3. Trụ cột Công nghệ</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>4. Trụ cột Vận hành</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>5. Trụ cột Văn hóa</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>6. Trụ cột Dữ liệu</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -732,7 +744,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -757,7 +769,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -782,7 +794,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -807,7 +819,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>
@@ -846,139 +858,139 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -1058,7 +1070,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -1140,7 +1152,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -1222,7 +1234,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -1304,7 +1316,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>
@@ -1400,52 +1412,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>DBI</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Hạng</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>DBI S1</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Hạng S1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DBI S2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Hạng S2</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>DBI S3</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Hạng S3</t>
         </is>
@@ -1646,44 +1658,44 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1. Trụ cột Khách hàng</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>2. Trụ cột Chiến lược</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>3. Trụ cột Công nghệ</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>4. Trụ cột Vận hành</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>5. Trụ cột Văn hóa</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>6. Trụ cột Dữ liệu</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -1708,7 +1720,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -1733,7 +1745,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -1758,7 +1770,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -1783,7 +1795,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>
@@ -1822,139 +1834,139 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ngân hàng</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -2036,7 +2048,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -2118,7 +2130,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -2200,7 +2212,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -2282,7 +2294,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>
@@ -2378,27 +2390,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Cách</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Kịch bản</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Mô tả</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Spearman vs cơ sở A</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ngân hàng đổi hạng</t>
         </is>
@@ -2603,34 +2615,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Hạng 1 (%)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Hạng 2 (%)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Hạng 3 (%)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Hạng 4 (%)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Hạng 5 (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Vietcombank</t>
         </is>
@@ -2652,7 +2664,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>BIDV</t>
         </is>
@@ -2674,7 +2686,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>VietinBank</t>
         </is>
@@ -2696,7 +2708,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
@@ -2718,7 +2730,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>TPBank</t>
         </is>

</xml_diff>